<commit_message>
Update catalogue data 2026-10-09T10:07:02.077Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1504,7 +1504,7 @@
         <v>3301 1651</v>
       </c>
       <c r="M27" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="28">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:03:02.959Z</v>
+        <v>2026-10-09T10:07:02.078Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:07:10.983Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -4169,7 +4169,7 @@
         <v>3301 1651</v>
       </c>
       <c r="M92" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="93">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:07:02.078Z</v>
+        <v>2026-10-09T10:07:10.989Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:07:18.167Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -10155,7 +10155,7 @@
         <v>3301 1651</v>
       </c>
       <c r="M238" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="239">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:07:10.989Z</v>
+        <v>2026-10-09T10:07:18.171Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:07:28.296Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -11508,7 +11508,7 @@
         <v>3301 1651</v>
       </c>
       <c r="M271" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="272">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:07:18.171Z</v>
+        <v>2026-10-09T10:07:28.301Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:07:40.384Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -7859,7 +7859,7 @@
         <v>3301 1651</v>
       </c>
       <c r="M182" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="183">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:07:28.301Z</v>
+        <v>2026-10-09T10:07:40.389Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:07:49.597Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -4415,7 +4415,7 @@
         <v>33011651</v>
       </c>
       <c r="M98" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="99">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:07:40.389Z</v>
+        <v>2026-10-09T10:07:49.601Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:08:01.173Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -3308,7 +3308,7 @@
         <v>66663444</v>
       </c>
       <c r="M71" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="72">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:07:49.601Z</v>
+        <v>2026-10-09T10:08:01.179Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:08:12.818Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -13148,7 +13148,7 @@
         <v>55858321</v>
       </c>
       <c r="M311" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="312">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:08:04.478Z</v>
+        <v>2026-10-09T10:08:12.823Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:08:22.866Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -3062,7 +3062,7 @@
         <v>70009001</v>
       </c>
       <c r="M65" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="66">
@@ -9868,7 +9868,7 @@
         <v>70009001</v>
       </c>
       <c r="M231" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="232">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:08:12.823Z</v>
+        <v>2026-10-09T10:08:22.871Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:08:42.032Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -2693,7 +2693,7 @@
         <v>66665266</v>
       </c>
       <c r="M56" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="57">
@@ -3103,7 +3103,7 @@
         <v>66665266</v>
       </c>
       <c r="M66" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="67">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:08:22.871Z</v>
+        <v>2026-10-09T10:08:42.037Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:08:50.028Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5727,7 +5727,7 @@
         <v>66665266</v>
       </c>
       <c r="M130" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="131">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:08:42.037Z</v>
+        <v>2026-10-09T10:08:50.034Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:08:58.168Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -7613,7 +7613,7 @@
         <v>66665266</v>
       </c>
       <c r="M176" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="177">
@@ -7818,7 +7818,7 @@
         <v>66665266</v>
       </c>
       <c r="M181" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="182">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:08:50.034Z</v>
+        <v>2026-10-09T10:08:58.170Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:09:05.175Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -13517,7 +13517,7 @@
         <v>66665266</v>
       </c>
       <c r="M320" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="321">
@@ -15690,7 +15690,7 @@
         <v>66665266</v>
       </c>
       <c r="M373" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="374">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:08:58.170Z</v>
+        <v>2026-10-09T10:09:05.179Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:09:25.212Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8064,7 +8064,7 @@
         <v>33663390</v>
       </c>
       <c r="M187" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="188">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:09:05.179Z</v>
+        <v>2026-10-09T10:09:25.217Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:09:37.280Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5440,7 +5440,7 @@
         <v>66600687</v>
       </c>
       <c r="M123" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="124">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:09:25.217Z</v>
+        <v>2026-10-09T10:09:37.285Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:10:08.437Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5431,7 +5431,7 @@
         <v>MOUHSINA AL SHAQAB</v>
       </c>
       <c r="J123" t="str">
-        <v>Al Yusufiya Arabians</v>
+        <v>Al Fuwairat Stud</v>
       </c>
       <c r="K123" t="str">
         <v>Aljamalstud.qr@gmail.com</v>
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:09:37.285Z</v>
+        <v>2026-10-09T10:10:08.442Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update catalogue data 2026-10-09T10:10:26.056Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1381,7 +1381,7 @@
         <v>55099688</v>
       </c>
       <c r="M24" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="25">
@@ -16488,7 +16488,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B1" t="str">
-        <v>2026-10-09T10:10:08.442Z</v>
+        <v>2026-10-09T10:10:26.062Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>